<commit_message>
adjust for import data excel
</commit_message>
<xml_diff>
--- a/inject_data.xlsx
+++ b/inject_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Works\THE RESONANZ\CODING\_WEBSITE\2026\luxury-guest-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCCCCBC4-DF9F-461D-A41D-F0059A806872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23C937C-1FF8-4C13-8BAE-ACDD836836FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14700" windowHeight="17385" xr2:uid="{45973840-4573-4F70-91D0-D6765A16B82F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{45973840-4573-4F70-91D0-D6765A16B82F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,17 +34,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>full_name</t>
   </si>
   <si>
-    <t>company</t>
-  </si>
-  <si>
-    <t>position</t>
-  </si>
-  <si>
     <t>seat_number</t>
   </si>
   <si>
@@ -54,10 +48,28 @@
     <t>PT. Example</t>
   </si>
   <si>
-    <t>Manager</t>
-  </si>
-  <si>
     <t>A-104</t>
+  </si>
+  <si>
+    <t>ga_so_position</t>
+  </si>
+  <si>
+    <t>phone_number</t>
+  </si>
+  <si>
+    <t>6281334178147</t>
+  </si>
+  <si>
+    <t>6287763127570</t>
+  </si>
+  <si>
+    <t>Percobaan</t>
+  </si>
+  <si>
+    <t>PT. Asik Sekali</t>
+  </si>
+  <si>
+    <t>X-92</t>
   </si>
 </sst>
 </file>
@@ -93,8 +105,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,35 +422,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FA8C1E6-A84E-478B-B16B-9EDC327A4A47}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adjust some function in send whatsapp, format template
</commit_message>
<xml_diff>
--- a/inject_data.xlsx
+++ b/inject_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Works\THE RESONANZ\CODING\_WEBSITE\2026\luxury-guest-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23C937C-1FF8-4C13-8BAE-ACDD836836FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCD2223-7AA6-446A-9D30-32531A1D8589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{45973840-4573-4F70-91D0-D6765A16B82F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>full_name</t>
   </si>
@@ -42,47 +42,41 @@
     <t>seat_number</t>
   </si>
   <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>PT. Example</t>
-  </si>
-  <si>
-    <t>A-104</t>
-  </si>
-  <si>
     <t>ga_so_position</t>
   </si>
   <si>
     <t>phone_number</t>
   </si>
   <si>
-    <t>6281334178147</t>
-  </si>
-  <si>
-    <t>6287763127570</t>
-  </si>
-  <si>
-    <t>Percobaan</t>
-  </si>
-  <si>
-    <t>PT. Asik Sekali</t>
-  </si>
-  <si>
-    <t>X-92</t>
+    <t>Giri</t>
+  </si>
+  <si>
+    <t>GAMAX001</t>
+  </si>
+  <si>
+    <t>Z-23</t>
+  </si>
+  <si>
+    <t>6281911016590</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,9 +99,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -433,42 +428,31 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="D3" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>